<commit_message>
Update for herindelingsverkiezingen 2026
</commit_message>
<xml_diff>
--- a/files/waarismijnstemlokaal.nl_invulformulier.xlsx
+++ b/files/waarismijnstemlokaal.nl_invulformulier.xlsx
@@ -3213,13 +3213,13 @@
     <t xml:space="preserve">YYYY-MM-DDTHH:MM:SS</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-18T07:30:00</t>
+    <t xml:space="preserve">2026-11-18T07:30:00</t>
   </si>
   <si>
     <t xml:space="preserve">Sluitingstijd</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-18T21:00:00</t>
+    <t xml:space="preserve">2026-11-18T21:00:00</t>
   </si>
   <si>
     <t xml:space="preserve">Toegankelijk voor mensen met een lichamelijke beperking</t>
@@ -3376,7 +3376,7 @@
     <t xml:space="preserve">Stembureaus &lt;verkiezing&gt; &lt;jaar&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">Stembureaus gemeenteraadsverkiezingen 2026</t>
+    <t xml:space="preserve">Stembureaus herindelingsverkiezingen 2026</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -3390,7 +3390,7 @@
     <t xml:space="preserve">NLODS&lt;CBS gemeentecode&gt;stembureaus&lt;YYYYMMDD&gt;&lt;oplopend getal van 000 t/m 999&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">NLODSGM0518stembureaus20260318017</t>
+    <t xml:space="preserve">NLODSGM0518stembureaus20261118018</t>
   </si>
   <si>
     <t xml:space="preserve">Omschrijving</t>
@@ -3403,7 +3403,7 @@
     <t xml:space="preserve">Overzicht van de locaties van stembureaus. De gegevens hebben betrekking op &lt;verkiezing&gt; op &lt;datum&gt;.</t>
   </si>
   <si>
-    <t xml:space="preserve">Overzicht van de locaties van stembureaus. De gegevens hebben betrekking op de Europese Parlementsverkiezingen op 18 maart 2026.</t>
+    <t xml:space="preserve">Overzicht van de locaties van stembureaus. De gegevens hebben betrekking op de herindelingsverkiezingen op 18 november 2026 waarbij de gemeenten Hilversum en Wijdemeren fuseren en verdergaan als de gemeente Hilversum.</t>
   </si>
   <si>
     <t xml:space="preserve">Eigenaar</t>
@@ -3442,7 +3442,7 @@
     <t xml:space="preserve">verkiezingen, stembureaus, overheid, democratie, stemmen, kiesdistrict, &lt;aard van de verkiezing&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">verkiezingen, stembureaus, overheid, democratie, stemmen, kiesdistrict, gemeenteraadsverkiezingen</t>
+    <t xml:space="preserve">verkiezingen, stembureaus, overheid, democratie, stemmen, kiesdistrict, herindelingsverkiezingen</t>
   </si>
   <si>
     <t xml:space="preserve">Thema</t>
@@ -3483,7 +3483,7 @@
     <t xml:space="preserve">YYYY-MM-DDTHH:MM:SS+-HH:MM</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-02-15T13:05:23+01:00</t>
+    <t xml:space="preserve">2026-10-15T13:05:23+01:00</t>
   </si>
   <si>
     <t xml:space="preserve">Relatie / gebruik andere standaarden</t>
@@ -3501,7 +3501,7 @@
     <t xml:space="preserve">YYYY-MM-DD</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-03-18</t>
+    <t xml:space="preserve">2026-11-18</t>
   </si>
   <si>
     <t xml:space="preserve">Update frequentie</t>
@@ -3513,7 +3513,7 @@
     <t xml:space="preserve">Incidenteel tot en met &lt;datum verkiezing&gt; (uiterste bekendmaking van stembureaus is 4 dagen voor de verkiezing)</t>
   </si>
   <si>
-    <t xml:space="preserve">Incidenteel tot en met 18 maart 2026 (uiterste bekendmaking van stembureaus is 4 dagen voor de verkiezingen)</t>
+    <t xml:space="preserve">Incidenteel tot en met 18 november 2026 (uiterste bekendmaking van stembureaus is 4 dagen voor de verkiezingen)</t>
   </si>
   <si>
     <t xml:space="preserve">Wijzigings datum</t>

</xml_diff>